<commit_message>
docs: reflejar contratos de Backoffice en el Excel de flujo de datos entregado
Mismos cambios que el .md: precio -> categoriaPrecio en eventos, aptoEventos
en locaciones, y las dos filas nuevas del catálogo de locaciones y la
tarifa de inscripción de Backoffice, en las filas de plantilla ya
estilizadas de la planilla.
</commit_message>
<xml_diff>
--- a/docs/05-entregas/Flujo de Datos - Modulo 6 - UADEnet.xlsx
+++ b/docs/05-entregas/Flujo de Datos - Modulo 6 - UADEnet.xlsx
@@ -616,12 +616,12 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>{"titulo": "string", "descripcion": "string", "locacionId": "uuid", "cupoMaximo": "number (entero &gt; 0)", "fechaInicio": "datetime ISO 8601", "fechaFin": "datetime ISO 8601 (posterior a fechaInicio)", "esPago": "boolean", "precio": "number (entero &gt; 0) | null — obligatorio si esPago = true"} — responde 409 si la locación ya tiene un evento solapado en ese rango horario</t>
+          <t>{"titulo": "string", "descripcion": "string", "locacionId": "uuid", "cupoMaximo": "number (entero &gt; 0)", "fechaInicio": "datetime ISO 8601", "fechaFin": "datetime ISO 8601 (posterior a fechaInicio)", "esPago": "boolean", "categoriaPrecio": "general | especial | null — obligatorio si esPago = true, resuelto contra la tarifa vigente de Backoffice"} — responde 409 si la locación ya tiene un evento solapado en ese rango horario, o si la locación no está aptoEventos</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>{"titulo": "Charla: Arquitectura de Software", "descripcion": "Charla abierta sobre patrones de arquitectura.", "locacionId": "c1a4e8d2-7b36-4f90-8e52-1d0a9c3b6f47", "cupoMaximo": 80, "fechaInicio": "2026-10-15T18:00:00-03:00", "fechaFin": "2026-10-15T20:00:00-03:00", "esPago": false, "precio": null}</t>
+          <t>{"titulo": "Charla: Arquitectura de Software", "descripcion": "Charla abierta sobre patrones de arquitectura.", "locacionId": "c1a4e8d2-7b36-4f90-8e52-1d0a9c3b6f47", "cupoMaximo": 80, "fechaInicio": "2026-10-15T18:00:00-03:00", "fechaFin": "2026-10-15T20:00:00-03:00", "esPago": false, "categoriaPrecio": null}</t>
         </is>
       </c>
     </row>
@@ -648,12 +648,12 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>[{"id": "uuid", "titulo": "string", "descripcion": "string", "locacionId": "uuid", "cupoMaximo": "number", "fechaInicio": "datetime", "fechaFin": "datetime", "esPago": "boolean", "precio": "number | null", "creadoPor": "string (id de usuario en CORE)", "locacion": {"nombre": "string", "sede": "string"}, "inscriptos": "number", "disponibles": "number", "yaInscripto": "boolean"}] — ordenado por fechaInicio. desde/hasta son ISO 8601 opcionales y filtran por solapamiento con la ventana. Locación resuelta y cupo calculado para el calendario de los portales; yaInscripto se calcula contra el usuario del JWT</t>
+          <t>[{"id": "uuid", "titulo": "string", "descripcion": "string", "locacionId": "uuid", "cupoMaximo": "number", "fechaInicio": "datetime", "fechaFin": "datetime", "esPago": "boolean", "categoriaPrecio": "general | especial | null", "creadoPor": "string (id de usuario en CORE)", "locacion": {"nombre": "string", "sede": "string"}, "inscriptos": "number", "disponibles": "number", "yaInscripto": "boolean"}] — ordenado por fechaInicio. desde/hasta son ISO 8601 opcionales y filtran por solapamiento con la ventana. Locación resuelta y cupo calculado para el calendario de los portales; yaInscripto se calcula contra el usuario del JWT</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>[{"id": "9f2b7c14-3d5a-4e88-9a10-6c2d5e7f1b03", "titulo": "Charla: Arquitectura de Software", "descripcion": "Charla abierta sobre patrones de arquitectura.", "locacionId": "c1a4e8d2-7b36-4f90-8e52-1d0a9c3b6f47", "cupoMaximo": 80, "fechaInicio": "2026-10-15T18:00:00-03:00", "fechaFin": "2026-10-15T20:00:00-03:00", "esPago": false, "precio": null, "creadoPor": "u-10432", "locacion": {"nombre": "Aula Magna", "sede": "Monserrat"}, "inscriptos": 63, "disponibles": 17, "yaInscripto": false}]</t>
+          <t>[{"id": "9f2b7c14-3d5a-4e88-9a10-6c2d5e7f1b03", "titulo": "Charla: Arquitectura de Software", "descripcion": "Charla abierta sobre patrones de arquitectura.", "locacionId": "c1a4e8d2-7b36-4f90-8e52-1d0a9c3b6f47", "cupoMaximo": 80, "fechaInicio": "2026-10-15T18:00:00-03:00", "fechaFin": "2026-10-15T20:00:00-03:00", "esPago": false, "categoriaPrecio": null, "creadoPor": "u-10432", "locacion": {"nombre": "Aula Magna", "sede": "Monserrat"}, "inscriptos": 63, "disponibles": 17, "yaInscripto": false, "precio": null}]</t>
         </is>
       </c>
     </row>
@@ -712,12 +712,12 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>[{"id": "uuid", "nombre": "string", "sede": "string", "capacidad": "number"}] — catálogo propio, no se integra con Backoffice Administrativo (decidido, ver integraciones.md)</t>
+          <t>[{"id": "uuid", "nombre": "string", "sede": "string", "capacidad": "number", "aptoEventos": "boolean"}] — catálogo sincronizado desde Backoffice Administrativo (ver ADR 0013)</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>[{"id": "c1a4e8d2-7b36-4f90-8e52-1d0a9c3b6f47", "nombre": "Aula Magna", "sede": "Monserrat", "capacidad": 120}]</t>
+          <t>[{"id": "c1a4e8d2-7b36-4f90-8e52-1d0a9c3b6f47", "nombre": "Aula Magna", "sede": "Monserrat", "capacidad": 120, "aptoEventos": true}]</t>
         </is>
       </c>
     </row>
@@ -1042,20 +1042,68 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="n"/>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Backoffice Administrativo</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Restful API</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>GET {BACKOFFICE_BASE_URL}/locaciones</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>[{"id": "uuid", "nombre": "string", "sede": "string", "capacidad": "number", "aptoEventos": "boolean"}] — catálogo de locaciones aptas para eventos, sincronizado periódicamente (ver ADR 0013)</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>[{"id": "c1a4e8d2-7b36-4f90-8e52-1d0a9c3b6f47", "nombre": "Aula Magna", "sede": "Monserrat", "capacidad": 120, "aptoEventos": true}]</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Backoffice Administrativo</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Restful API</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>GET {BACKOFFICE_BASE_URL}/tarifas/evento-inscripcion/{categoria}</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>{"categoria": "general | especial", "monto": "number (entero, en pesos)"} — tarifa vigente para esa categoría; se consulta al listar eventos y al confirmar cada inscripción paga</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>{"categoria": "especial", "monto": 12500}</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n"/>

</xml_diff>